<commit_message>
Add S1 3PL fit script and S1 results
Add a new analysis script for Simulado_I (Piaui/2026/Programas/Fit_3PL_Fix_2EM_MT_S1.R) that fits a 3PL model with some item parameters fixed, writes SAEB-scaled outputs and generates diagnostic PDFs. Update .Rhistory to point to Simulado_I and to use the df_1ª_SIMULA RDS and gabarito_1ª SIMULA file, and change several output filenames to S1. Add generated result files (xlsx and pdf) under ResultadosTRI_2EM_MT/Simulado_I. Minor change in the existing S2 script to disable rounding of TabItens. Update the gabarito_2serie_mt 1ª SIMULA.xlsx in Dados.
</commit_message>
<xml_diff>
--- a/Piaui/2026/ResultadosTRI_2EM_MT/Simulado_II/EstItens_2EM_MT_S2.xlsx
+++ b/Piaui/2026/ResultadosTRI_2EM_MT/Simulado_II/EstItens_2EM_MT_S2.xlsx
@@ -473,19 +473,19 @@
         <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>1.014</v>
+        <v>1.01438425</v>
       </c>
       <c r="C2" t="n">
-        <v>0.968</v>
+        <v>0.968467999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02</v>
+        <v>0.020287685</v>
       </c>
       <c r="E2" t="n">
-        <v>298.423</v>
+        <v>298.4234</v>
       </c>
       <c r="F2" t="n">
-        <v>0.023</v>
+        <v>0.0234630000000001</v>
       </c>
       <c r="G2" t="s">
         <v>8</v>
@@ -496,19 +496,19 @@
         <v>9</v>
       </c>
       <c r="B3" t="n">
-        <v>0.538</v>
+        <v>0.538477099999999</v>
       </c>
       <c r="C3" t="n">
-        <v>3.985</v>
+        <v>3.985406</v>
       </c>
       <c r="D3" t="n">
-        <v>0.011</v>
+        <v>0.010769542</v>
       </c>
       <c r="E3" t="n">
-        <v>449.27</v>
+        <v>449.2703</v>
       </c>
       <c r="F3" t="n">
-        <v>0.073</v>
+        <v>0.0732108400000002</v>
       </c>
       <c r="G3" t="s">
         <v>8</v>
@@ -519,19 +519,19 @@
         <v>10</v>
       </c>
       <c r="B4" t="n">
-        <v>1.678</v>
+        <v>1.67842839937054</v>
       </c>
       <c r="C4" t="n">
-        <v>3.337</v>
+        <v>3.33746179479017</v>
       </c>
       <c r="D4" t="n">
-        <v>0.034</v>
+        <v>0.0335685679874107</v>
       </c>
       <c r="E4" t="n">
-        <v>416.873</v>
+        <v>416.873089739509</v>
       </c>
       <c r="F4" t="n">
-        <v>0.224</v>
+        <v>0.223774125614892</v>
       </c>
       <c r="G4" t="s">
         <v>11</v>
@@ -542,19 +542,19 @@
         <v>12</v>
       </c>
       <c r="B5" t="n">
-        <v>0.843</v>
+        <v>0.843417332943628</v>
       </c>
       <c r="C5" t="n">
-        <v>1.013</v>
+        <v>1.01328778238753</v>
       </c>
       <c r="D5" t="n">
-        <v>0.017</v>
+        <v>0.0168683466588725</v>
       </c>
       <c r="E5" t="n">
-        <v>300.664</v>
+        <v>300.664389119377</v>
       </c>
       <c r="F5" t="n">
-        <v>0.016</v>
+        <v>0.0161555405979066</v>
       </c>
       <c r="G5" t="s">
         <v>11</v>
@@ -565,19 +565,19 @@
         <v>13</v>
       </c>
       <c r="B6" t="n">
-        <v>1.098</v>
+        <v>1.09759810346949</v>
       </c>
       <c r="C6" t="n">
-        <v>1.389</v>
+        <v>1.3892371341247</v>
       </c>
       <c r="D6" t="n">
-        <v>0.022</v>
+        <v>0.0219519620693897</v>
       </c>
       <c r="E6" t="n">
-        <v>319.462</v>
+        <v>319.461856706235</v>
       </c>
       <c r="F6" t="n">
-        <v>0.009</v>
+        <v>0.00861415438945763</v>
       </c>
       <c r="G6" t="s">
         <v>11</v>
@@ -588,19 +588,19 @@
         <v>14</v>
       </c>
       <c r="B7" t="n">
-        <v>2.447</v>
+        <v>2.44728227192752</v>
       </c>
       <c r="C7" t="n">
-        <v>2.641</v>
+        <v>2.64058329223122</v>
       </c>
       <c r="D7" t="n">
-        <v>0.049</v>
+        <v>0.0489456454385505</v>
       </c>
       <c r="E7" t="n">
-        <v>382.029</v>
+        <v>382.029164611561</v>
       </c>
       <c r="F7" t="n">
-        <v>0.273</v>
+        <v>0.273345980545672</v>
       </c>
       <c r="G7" t="s">
         <v>11</v>
@@ -611,19 +611,19 @@
         <v>15</v>
       </c>
       <c r="B8" t="n">
-        <v>1.355</v>
+        <v>1.3550061182195</v>
       </c>
       <c r="C8" t="n">
-        <v>3.324</v>
+        <v>3.32413964940511</v>
       </c>
       <c r="D8" t="n">
-        <v>0.027</v>
+        <v>0.0271001223643901</v>
       </c>
       <c r="E8" t="n">
-        <v>416.207</v>
+        <v>416.206982470256</v>
       </c>
       <c r="F8" t="n">
-        <v>0.149</v>
+        <v>0.148654404061939</v>
       </c>
       <c r="G8" t="s">
         <v>11</v>
@@ -634,19 +634,19 @@
         <v>16</v>
       </c>
       <c r="B9" t="n">
-        <v>0.917</v>
+        <v>0.916616907137823</v>
       </c>
       <c r="C9" t="n">
-        <v>2.242</v>
+        <v>2.24238514226319</v>
       </c>
       <c r="D9" t="n">
-        <v>0.018</v>
+        <v>0.0183323381427565</v>
       </c>
       <c r="E9" t="n">
-        <v>362.119</v>
+        <v>362.11925711316</v>
       </c>
       <c r="F9" t="n">
-        <v>0.044</v>
+        <v>0.0438297978035109</v>
       </c>
       <c r="G9" t="s">
         <v>11</v>
@@ -657,19 +657,19 @@
         <v>17</v>
       </c>
       <c r="B10" t="n">
-        <v>1.227</v>
+        <v>1.22746389198006</v>
       </c>
       <c r="C10" t="n">
-        <v>2.443</v>
+        <v>2.44251074785695</v>
       </c>
       <c r="D10" t="n">
-        <v>0.025</v>
+        <v>0.0245492778396012</v>
       </c>
       <c r="E10" t="n">
-        <v>372.126</v>
+        <v>372.125537392847</v>
       </c>
       <c r="F10" t="n">
-        <v>0.189</v>
+        <v>0.188631300475902</v>
       </c>
       <c r="G10" t="s">
         <v>11</v>
@@ -680,19 +680,19 @@
         <v>18</v>
       </c>
       <c r="B11" t="n">
-        <v>1.945</v>
+        <v>1.94464688431503</v>
       </c>
       <c r="C11" t="n">
-        <v>2.989</v>
+        <v>2.98888831515384</v>
       </c>
       <c r="D11" t="n">
-        <v>0.039</v>
+        <v>0.0388929376863006</v>
       </c>
       <c r="E11" t="n">
-        <v>399.444</v>
+        <v>399.444415757692</v>
       </c>
       <c r="F11" t="n">
-        <v>0.275</v>
+        <v>0.275302279751138</v>
       </c>
       <c r="G11" t="s">
         <v>11</v>
@@ -703,19 +703,19 @@
         <v>19</v>
       </c>
       <c r="B12" t="n">
-        <v>0.519</v>
+        <v>0.519475067516627</v>
       </c>
       <c r="C12" t="n">
-        <v>2.407</v>
+        <v>2.40745609035654</v>
       </c>
       <c r="D12" t="n">
-        <v>0.01</v>
+        <v>0.0103895013503325</v>
       </c>
       <c r="E12" t="n">
-        <v>370.373</v>
+        <v>370.372804517827</v>
       </c>
       <c r="F12" t="n">
-        <v>0.015</v>
+        <v>0.0152774627783021</v>
       </c>
       <c r="G12" t="s">
         <v>11</v>
@@ -726,19 +726,19 @@
         <v>20</v>
       </c>
       <c r="B13" t="n">
-        <v>1.419</v>
+        <v>1.41929765393194</v>
       </c>
       <c r="C13" t="n">
-        <v>2.015</v>
+        <v>2.01549611142795</v>
       </c>
       <c r="D13" t="n">
-        <v>0.028</v>
+        <v>0.0283859530786387</v>
       </c>
       <c r="E13" t="n">
-        <v>350.775</v>
+        <v>350.774805571398</v>
       </c>
       <c r="F13" t="n">
-        <v>0.107</v>
+        <v>0.10712038442481</v>
       </c>
       <c r="G13" t="s">
         <v>11</v>
@@ -749,19 +749,19 @@
         <v>21</v>
       </c>
       <c r="B14" t="n">
-        <v>2.324</v>
+        <v>2.3242653531958</v>
       </c>
       <c r="C14" t="n">
-        <v>2.814</v>
+        <v>2.81373560338526</v>
       </c>
       <c r="D14" t="n">
-        <v>0.046</v>
+        <v>0.046485307063916</v>
       </c>
       <c r="E14" t="n">
-        <v>390.687</v>
+        <v>390.686780169263</v>
       </c>
       <c r="F14" t="n">
-        <v>0.126</v>
+        <v>0.125612831543424</v>
       </c>
       <c r="G14" t="s">
         <v>11</v>
@@ -772,19 +772,19 @@
         <v>22</v>
       </c>
       <c r="B15" t="n">
-        <v>1.019</v>
+        <v>1.01910811933425</v>
       </c>
       <c r="C15" t="n">
-        <v>2.253</v>
+        <v>2.25285085200418</v>
       </c>
       <c r="D15" t="n">
-        <v>0.02</v>
+        <v>0.0203821623866851</v>
       </c>
       <c r="E15" t="n">
-        <v>362.643</v>
+        <v>362.642542600209</v>
       </c>
       <c r="F15" t="n">
-        <v>0.134</v>
+        <v>0.133717628186471</v>
       </c>
       <c r="G15" t="s">
         <v>11</v>
@@ -795,16 +795,16 @@
         <v>23</v>
       </c>
       <c r="B16" t="n">
-        <v>3.1</v>
+        <v>3.09999999999999</v>
       </c>
       <c r="C16" t="n">
-        <v>2.907</v>
+        <v>2.90738000000001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.062</v>
+        <v>0.0619999999999999</v>
       </c>
       <c r="E16" t="n">
-        <v>395.369</v>
+        <v>395.369000000001</v>
       </c>
       <c r="F16" t="n">
         <v>0.294</v>
@@ -818,19 +818,19 @@
         <v>24</v>
       </c>
       <c r="B17" t="n">
-        <v>2.297</v>
+        <v>2.29711405752564</v>
       </c>
       <c r="C17" t="n">
-        <v>3.13</v>
+        <v>3.13047367299297</v>
       </c>
       <c r="D17" t="n">
-        <v>0.046</v>
+        <v>0.0459422811505127</v>
       </c>
       <c r="E17" t="n">
-        <v>406.524</v>
+        <v>406.523683649649</v>
       </c>
       <c r="F17" t="n">
-        <v>0.19</v>
+        <v>0.190059005006648</v>
       </c>
       <c r="G17" t="s">
         <v>11</v>
@@ -841,19 +841,19 @@
         <v>25</v>
       </c>
       <c r="B18" t="n">
-        <v>2.151</v>
+        <v>2.15103942755705</v>
       </c>
       <c r="C18" t="n">
-        <v>2.382</v>
+        <v>2.3817324886393</v>
       </c>
       <c r="D18" t="n">
-        <v>0.043</v>
+        <v>0.0430207885511409</v>
       </c>
       <c r="E18" t="n">
-        <v>369.087</v>
+        <v>369.086624431965</v>
       </c>
       <c r="F18" t="n">
-        <v>0.242</v>
+        <v>0.242316659107945</v>
       </c>
       <c r="G18" t="s">
         <v>11</v>
@@ -864,19 +864,19 @@
         <v>26</v>
       </c>
       <c r="B19" t="n">
-        <v>1.797</v>
+        <v>1.79703232190086</v>
       </c>
       <c r="C19" t="n">
-        <v>3.408</v>
+        <v>3.40840452206764</v>
       </c>
       <c r="D19" t="n">
-        <v>0.036</v>
+        <v>0.0359406464380172</v>
       </c>
       <c r="E19" t="n">
-        <v>420.42</v>
+        <v>420.420226103382</v>
       </c>
       <c r="F19" t="n">
-        <v>0.173</v>
+        <v>0.173284858666627</v>
       </c>
       <c r="G19" t="s">
         <v>11</v>
@@ -887,19 +887,19 @@
         <v>27</v>
       </c>
       <c r="B20" t="n">
-        <v>3.183</v>
+        <v>3.18303381498567</v>
       </c>
       <c r="C20" t="n">
-        <v>3.063</v>
+        <v>3.06291855416498</v>
       </c>
       <c r="D20" t="n">
-        <v>0.064</v>
+        <v>0.0636606762997134</v>
       </c>
       <c r="E20" t="n">
-        <v>403.146</v>
+        <v>403.145927708249</v>
       </c>
       <c r="F20" t="n">
-        <v>0.226</v>
+        <v>0.226194567654401</v>
       </c>
       <c r="G20" t="s">
         <v>11</v>
@@ -913,7 +913,7 @@
         <v>2.45</v>
       </c>
       <c r="C21" t="n">
-        <v>2.901</v>
+        <v>2.90072</v>
       </c>
       <c r="D21" t="n">
         <v>0.049</v>
@@ -933,19 +933,19 @@
         <v>29</v>
       </c>
       <c r="B22" t="n">
-        <v>2.138</v>
+        <v>2.13837090667299</v>
       </c>
       <c r="C22" t="n">
-        <v>3.203</v>
+        <v>3.20256321394018</v>
       </c>
       <c r="D22" t="n">
-        <v>0.043</v>
+        <v>0.0427674181334598</v>
       </c>
       <c r="E22" t="n">
-        <v>410.128</v>
+        <v>410.128160697009</v>
       </c>
       <c r="F22" t="n">
-        <v>0.293</v>
+        <v>0.292881758190988</v>
       </c>
       <c r="G22" t="s">
         <v>11</v>
@@ -956,19 +956,19 @@
         <v>30</v>
       </c>
       <c r="B23" t="n">
-        <v>1.476</v>
+        <v>1.47638096576423</v>
       </c>
       <c r="C23" t="n">
-        <v>4.141</v>
+        <v>4.14137140122663</v>
       </c>
       <c r="D23" t="n">
-        <v>0.03</v>
+        <v>0.0295276193152846</v>
       </c>
       <c r="E23" t="n">
-        <v>457.069</v>
+        <v>457.068570061332</v>
       </c>
       <c r="F23" t="n">
-        <v>0.118</v>
+        <v>0.118216094227102</v>
       </c>
       <c r="G23" t="s">
         <v>11</v>
@@ -979,19 +979,19 @@
         <v>31</v>
       </c>
       <c r="B24" t="n">
-        <v>0.496</v>
+        <v>0.495925387562008</v>
       </c>
       <c r="C24" t="n">
-        <v>3.999</v>
+        <v>3.99929564686165</v>
       </c>
       <c r="D24" t="n">
-        <v>0.01</v>
+        <v>0.00991850775124017</v>
       </c>
       <c r="E24" t="n">
-        <v>449.965</v>
+        <v>449.964782343082</v>
       </c>
       <c r="F24" t="n">
-        <v>0.121</v>
+        <v>0.120663536401756</v>
       </c>
       <c r="G24" t="s">
         <v>11</v>
@@ -1002,19 +1002,19 @@
         <v>32</v>
       </c>
       <c r="B25" t="n">
-        <v>1.705</v>
+        <v>1.70485770995118</v>
       </c>
       <c r="C25" t="n">
-        <v>2.214</v>
+        <v>2.21387696226408</v>
       </c>
       <c r="D25" t="n">
-        <v>0.034</v>
+        <v>0.0340971541990235</v>
       </c>
       <c r="E25" t="n">
-        <v>360.694</v>
+        <v>360.693848113204</v>
       </c>
       <c r="F25" t="n">
-        <v>0.175</v>
+        <v>0.174632413573961</v>
       </c>
       <c r="G25" t="s">
         <v>11</v>
@@ -1025,19 +1025,19 @@
         <v>33</v>
       </c>
       <c r="B26" t="n">
-        <v>1.247</v>
+        <v>1.24657501230464</v>
       </c>
       <c r="C26" t="n">
-        <v>1.855</v>
+        <v>1.85487257458894</v>
       </c>
       <c r="D26" t="n">
-        <v>0.025</v>
+        <v>0.0249315002460928</v>
       </c>
       <c r="E26" t="n">
-        <v>342.744</v>
+        <v>342.743628729447</v>
       </c>
       <c r="F26" t="n">
-        <v>0.104</v>
+        <v>0.103844749041497</v>
       </c>
       <c r="G26" t="s">
         <v>11</v>
@@ -1048,19 +1048,19 @@
         <v>34</v>
       </c>
       <c r="B27" t="n">
-        <v>1.227</v>
+        <v>1.22742731801846</v>
       </c>
       <c r="C27" t="n">
-        <v>2.673</v>
+        <v>2.67255617837511</v>
       </c>
       <c r="D27" t="n">
-        <v>0.025</v>
+        <v>0.0245485463603693</v>
       </c>
       <c r="E27" t="n">
-        <v>383.628</v>
+        <v>383.627808918756</v>
       </c>
       <c r="F27" t="n">
-        <v>0.194</v>
+        <v>0.193535074744008</v>
       </c>
       <c r="G27" t="s">
         <v>11</v>

</xml_diff>